<commit_message>
D-R6 draft: 20 dBm e.i.r.p. via adaptive FHSS + LBT for SRI/MRM (CNAF UN-85 a, EN 300 328)
- linkbudget: S24-S26 (SP4 + omni at 20 dBm while hopping; worst RF_PWR step), FHSS goodput
- workbook rebuilt: 26 scenarios, FHSS block in Throughput, UN-85 a) row; 0 dB diff vs Python
- phy_config: TEAM_FHSS profile, 29-channel hop set clear of the other teams, EN 300 328 checks
- fw: power cap per profile, nrf24_cca (RPD), hop-set-only channels, 50 ms COT + idle gap; 194 checks
- sim: --fhss radio layer (25 ms hops, CCA, busy hops skipped, re-sync); T12/T13, 13/13 pass
- docs: DECISIONS D-R6, TEST_PLAN v0.4 (T0 all steps, T17, T18), Atenea Q3 rewritten, handoff v0.4

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MU9yLRr2JqK4PHEE7hWEta
</commit_message>
<xml_diff>
--- a/radio/MTP-F26_TeamC_Radio_LinkBudget.xlsx
+++ b/radio/MTP-F26_TeamC_Radio_LinkBudget.xlsx
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -163,6 +163,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -552,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -585,126 +586,133 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Link Budget - AN5142 rows (course-corrected), one column per scenario S1-S12. This is the ANNEX 'Link Budget Analysis' artefact.</t>
+          <t>Link Budget - AN5142 rows (course-corrected), one column per scenario S1-S26. This is the ANNEX 'Link Budget Analysis' artefact.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Height Sweep - same budgets recomputed for antenna heights 0.5-1.5 m.</t>
+          <t>S21-S23 = 2.4 GHz baseline (E01-ML01SP4 + one omni, 10 mW e.i.r.p.). S24-S26 = D-R6 draft: same hardware as adaptive FHSS + LBT at 20 dBm e.i.r.p. (UN-85 a), only if Atenea Q3 = yes.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Throughput - lines delivered in 120 s per radio/data rate; occupied bandwidth check for the 250 kHz 868 sub-band.</t>
+          <t>Height Sweep - same budgets recomputed for antenna heights 0.5-1.5 m.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Candidates - radio module shortlist with datasheet figures, gotchas and compliance notes.</t>
+          <t>Throughput - lines delivered in 120 s per radio/data rate; occupied bandwidth check for the 250 kHz 868 sub-band.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Candidates - radio module shortlist with datasheet figures, gotchas and compliance notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Regulatory - CNAF 2017 bands usable for a 2-minute continuous round.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Legend</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Blue text = input you may change. Black = formula. Green = link to another sheet.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Yellow fill = key assumption that must be replaced by a measurement (antenna gain in box, container loss, multipath, heights).</t>
+          <t>Blue text = input you may change. Black = formula. Green = link to another sheet.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Yellow fill = key assumption that must be replaced by a measurement (antenna gain in box, container loss, multipath, heights).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Green fill = results.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Model</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>P_R = EIRP + L_FS + L_GB + L0 + LMP + LObs + G_R + LConR. L_GB = 10log10(1 + a² - 2a|cos(2πΔd/λ)|): the course correction removes AN5142's 1/2 factor.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Beyond the breakpoint (x &lt; π/2) loss grows 40 dB/decade and is almost frequency-independent: antenna HEIGHT, TX power and RX sensitivity decide the link.</t>
+          <t>P_R = EIRP + L_FS + L_GB + L0 + LMP + LObs + G_R + LConR. L_GB = 10log10(1 + a² - 2a|cos(2πΔd/λ)|): the course correction removes AN5142's 1/2 factor.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>Beyond the breakpoint (x &lt; π/2) loss grows 40 dB/decade and is almost frequency-independent: antenna HEIGHT, TX power and RX sensitivity decide the link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>In the interference zone the |cos| envelope produces artificial nulls; real links fade between -∞ and +6 dB there. Measure.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>How to use</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>1. Change blue cells in 'Link Budget' (e.g. antenna gain after measuring), read the margin rows.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2. The same model is in radio/linkbudget.py for quick what-ifs; radio/build_workbook.py regenerates this file.</t>
+          <t>1. Change blue cells in 'Link Budget' (e.g. antenna gain after measuring), read the margin rows.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2. The same model is in radio/linkbudget.py for quick what-ifs; radio/build_workbook.py regenerates this file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>3. Replace every yellow assumption with a measured value (tests T2 bench PER, T4/T5 range, T13 spectrum).</t>
         </is>
@@ -721,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA84"/>
+  <dimension ref="A1:AD87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -751,6 +759,9 @@
     <col width="17" customWidth="1" min="25" max="25"/>
     <col width="17" customWidth="1" min="26" max="26"/>
     <col width="17" customWidth="1" min="27" max="27"/>
+    <col width="17" customWidth="1" min="28" max="28"/>
+    <col width="17" customWidth="1" min="29" max="29"/>
+    <col width="17" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -901,6 +912,21 @@
       <c r="AA3" s="5" t="inlineStr">
         <is>
           <t>S23</t>
+        </is>
+      </c>
+      <c r="AB3" s="5" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="AC3" s="5" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="AD3" s="5" t="inlineStr">
+        <is>
+          <t>S26</t>
         </is>
       </c>
     </row>
@@ -936,6 +962,9 @@
       <c r="Y4" s="7" t="n"/>
       <c r="Z4" s="7" t="n"/>
       <c r="AA4" s="7" t="n"/>
+      <c r="AB4" s="7" t="n"/>
+      <c r="AC4" s="7" t="n"/>
+      <c r="AD4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1063,6 +1092,21 @@
       <c r="AA5" s="8" t="inlineStr">
         <is>
           <t>NM hop 100 m</t>
+        </is>
+      </c>
+      <c r="AB5" s="8" t="inlineStr">
+        <is>
+          <t>SRI 70 m</t>
+        </is>
+      </c>
+      <c r="AC5" s="8" t="inlineStr">
+        <is>
+          <t>MRM 260 m</t>
+        </is>
+      </c>
+      <c r="AD5" s="8" t="inlineStr">
+        <is>
+          <t>MRM 260 m</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1216,7 @@
       </c>
       <c r="X6" s="8" t="inlineStr">
         <is>
-          <t>E01-ML01DP5 2.4G | 250 kbps, 100 mW FHSS (if Atenea Q3 = yes)</t>
+          <t>E01-ML01DP5 2.4G | 250 kbps, 100 mW FHSS (DP5, superseded by S25)</t>
         </is>
       </c>
       <c r="Y6" s="8" t="inlineStr">
@@ -1188,6 +1232,21 @@
       <c r="AA6" s="8" t="inlineStr">
         <is>
           <t>E01-ML01SP4 2.4G | 250 kbps, -10 dB obstr., omni (2.4 baseline)</t>
+        </is>
+      </c>
+      <c r="AB6" s="8" t="inlineStr">
+        <is>
+          <t>E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (D-R6)</t>
+        </is>
+      </c>
+      <c r="AC6" s="8" t="inlineStr">
+        <is>
+          <t>E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (D-R6)</t>
+        </is>
+      </c>
+      <c r="AD6" s="8" t="inlineStr">
+        <is>
+          <t>E01-ML01SP4 2.4G | 250 kbps, omni, FHSS worst RF_PWR step (D-R6)</t>
         </is>
       </c>
     </row>
@@ -1279,6 +1338,15 @@
         <v>250</v>
       </c>
       <c r="AA7" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="AB7" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="AC7" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="AD7" s="9" t="n">
         <v>250</v>
       </c>
     </row>
@@ -1292,7 +1360,7 @@
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>868: e.r.p. (UN-39); 2.4 GHz: e.i.r.p. (UN-85 b)</t>
+          <t>868: e.r.p. (UN-39); 2.4 GHz: e.i.r.p. (UN-85 b; FHSS UN-85 a)</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -1406,6 +1474,21 @@
         </is>
       </c>
       <c r="AA8" s="10" t="inlineStr">
+        <is>
+          <t>EIRP</t>
+        </is>
+      </c>
+      <c r="AB8" s="10" t="inlineStr">
+        <is>
+          <t>EIRP</t>
+        </is>
+      </c>
+      <c r="AC8" s="10" t="inlineStr">
+        <is>
+          <t>EIRP</t>
+        </is>
+      </c>
+      <c r="AD8" s="10" t="inlineStr">
         <is>
           <t>EIRP</t>
         </is>
@@ -1429,7 +1512,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>500 mW e.r.p. = 27 dBm; 10 mW e.i.r.p. = 10 dBm</t>
+          <t>500 mW e.r.p. = 27 dBm; 10 mW e.i.r.p. = 10 dBm; FHSS 100 mW = 20 dBm</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
@@ -1500,6 +1583,15 @@
       </c>
       <c r="AA9" s="11" t="n">
         <v>10</v>
+      </c>
+      <c r="AB9" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="AC9" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="AD9" s="11" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -1534,6 +1626,9 @@
       <c r="Y10" s="7" t="n"/>
       <c r="Z10" s="7" t="n"/>
       <c r="AA10" s="7" t="n"/>
+      <c r="AB10" s="7" t="n"/>
+      <c r="AC10" s="7" t="n"/>
+      <c r="AD10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1625,6 +1720,15 @@
       <c r="AA11" s="12" t="n">
         <v>2440</v>
       </c>
+      <c r="AB11" s="12" t="n">
+        <v>2441</v>
+      </c>
+      <c r="AC11" s="12" t="n">
+        <v>2441</v>
+      </c>
+      <c r="AD11" s="12" t="n">
+        <v>2441</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1716,6 +1820,15 @@
       <c r="AA12" s="13" t="n">
         <v>299792458</v>
       </c>
+      <c r="AB12" s="13" t="n">
+        <v>299792458</v>
+      </c>
+      <c r="AC12" s="13" t="n">
+        <v>299792458</v>
+      </c>
+      <c r="AD12" s="13" t="n">
+        <v>299792458</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1828,6 +1941,18 @@
       </c>
       <c r="AA13" s="14">
         <f>AA12/(AA11*1000000)</f>
+        <v/>
+      </c>
+      <c r="AB13" s="14">
+        <f>AB12/(AB11*1000000)</f>
+        <v/>
+      </c>
+      <c r="AC13" s="14">
+        <f>AC12/(AC11*1000000)</f>
+        <v/>
+      </c>
+      <c r="AD13" s="14">
+        <f>AD12/(AD11*1000000)</f>
         <v/>
       </c>
     </row>
@@ -1863,6 +1988,9 @@
       <c r="Y14" s="7" t="n"/>
       <c r="Z14" s="7" t="n"/>
       <c r="AA14" s="7" t="n"/>
+      <c r="AB14" s="7" t="n"/>
+      <c r="AC14" s="7" t="n"/>
+      <c r="AD14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1954,6 +2082,15 @@
       <c r="AA15" s="11" t="n">
         <v>7</v>
       </c>
+      <c r="AB15" s="11" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="AC15" s="11" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="AD15" s="11" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2045,6 +2182,15 @@
       <c r="AA16" s="11" t="n">
         <v>0</v>
       </c>
+      <c r="AB16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD16" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2136,6 +2282,15 @@
       <c r="AA17" s="11" t="n">
         <v>-0.5</v>
       </c>
+      <c r="AB17" s="11" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="AC17" s="11" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="AD17" s="11" t="n">
+        <v>-0.5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2250,6 +2405,18 @@
         <f>AA15+AA16+AA17</f>
         <v/>
       </c>
+      <c r="AB18" s="15">
+        <f>AB15+AB16+AB17</f>
+        <v/>
+      </c>
+      <c r="AC18" s="15">
+        <f>AC15+AC16+AC17</f>
+        <v/>
+      </c>
+      <c r="AD18" s="15">
+        <f>AD15+AD16+AD17</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2341,6 +2508,15 @@
       <c r="AA19" s="16" t="n">
         <v>2</v>
       </c>
+      <c r="AB19" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC19" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD19" s="16" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2455,6 +2631,18 @@
         <f>AA18+AA19</f>
         <v/>
       </c>
+      <c r="AB20" s="15">
+        <f>AB18+AB19</f>
+        <v/>
+      </c>
+      <c r="AC20" s="15">
+        <f>AC18+AC19</f>
+        <v/>
+      </c>
+      <c r="AD20" s="15">
+        <f>AD18+AD19</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2567,6 +2755,18 @@
       </c>
       <c r="AA21" s="15">
         <f>AA20-2.15</f>
+        <v/>
+      </c>
+      <c r="AB21" s="15">
+        <f>AB20-2.15</f>
+        <v/>
+      </c>
+      <c r="AC21" s="15">
+        <f>AC20-2.15</f>
+        <v/>
+      </c>
+      <c r="AD21" s="15">
+        <f>AD20-2.15</f>
         <v/>
       </c>
     </row>
@@ -2673,6 +2873,18 @@
       </c>
       <c r="AA22" s="17">
         <f>IF(IF(AA8="ERP",AA21,AA20)&lt;=AA9,"OK","OVER LIMIT")</f>
+        <v/>
+      </c>
+      <c r="AB22" s="17">
+        <f>IF(IF(AB8="ERP",AB21,AB20)&lt;=AB9,"OK","OVER LIMIT")</f>
+        <v/>
+      </c>
+      <c r="AC22" s="17">
+        <f>IF(IF(AC8="ERP",AC21,AC20)&lt;=AC9,"OK","OVER LIMIT")</f>
+        <v/>
+      </c>
+      <c r="AD22" s="17">
+        <f>IF(IF(AD8="ERP",AD21,AD20)&lt;=AD9,"OK","OVER LIMIT")</f>
         <v/>
       </c>
     </row>
@@ -2708,6 +2920,9 @@
       <c r="Y23" s="7" t="n"/>
       <c r="Z23" s="7" t="n"/>
       <c r="AA23" s="7" t="n"/>
+      <c r="AB23" s="7" t="n"/>
+      <c r="AC23" s="7" t="n"/>
+      <c r="AD23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2795,6 +3010,15 @@
       <c r="AA24" s="13" t="n">
         <v>100</v>
       </c>
+      <c r="AB24" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="AC24" s="13" t="n">
+        <v>260</v>
+      </c>
+      <c r="AD24" s="13" t="n">
+        <v>260</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2884,6 +3108,15 @@
         <v>0.75</v>
       </c>
       <c r="AA25" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AB25" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AC25" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AD25" s="18" t="n">
         <v>0.75</v>
       </c>
     </row>
@@ -2973,6 +3206,15 @@
       <c r="AA26" s="18" t="n">
         <v>0.75</v>
       </c>
+      <c r="AB26" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AC26" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AD26" s="18" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3064,6 +3306,15 @@
       <c r="AA27" s="19" t="n">
         <v>1</v>
       </c>
+      <c r="AB27" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC27" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD27" s="19" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3178,6 +3429,18 @@
         <f>SQRT(AA24^2+(AA25+AA26)^2)-SQRT(AA24^2+(AA25-AA26)^2)</f>
         <v/>
       </c>
+      <c r="AB28" s="20">
+        <f>SQRT(AB24^2+(AB25+AB26)^2)-SQRT(AB24^2+(AB25-AB26)^2)</f>
+        <v/>
+      </c>
+      <c r="AC28" s="20">
+        <f>SQRT(AC24^2+(AC25+AC26)^2)-SQRT(AC24^2+(AC25-AC26)^2)</f>
+        <v/>
+      </c>
+      <c r="AD28" s="20">
+        <f>SQRT(AD24^2+(AD25+AD26)^2)-SQRT(AD24^2+(AD25-AD26)^2)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3290,6 +3553,18 @@
       </c>
       <c r="AA29" s="21">
         <f>2*PI()*AA28/AA13</f>
+        <v/>
+      </c>
+      <c r="AB29" s="21">
+        <f>2*PI()*AB28/AB13</f>
+        <v/>
+      </c>
+      <c r="AC29" s="21">
+        <f>2*PI()*AC28/AC13</f>
+        <v/>
+      </c>
+      <c r="AD29" s="21">
+        <f>2*PI()*AD28/AD13</f>
         <v/>
       </c>
     </row>
@@ -3398,6 +3673,18 @@
         <f>IF(AA29&lt;PI()/2,"beyond breakpoint","interference zone")</f>
         <v/>
       </c>
+      <c r="AB30" s="17">
+        <f>IF(AB29&lt;PI()/2,"beyond breakpoint","interference zone")</f>
+        <v/>
+      </c>
+      <c r="AC30" s="17">
+        <f>IF(AC29&lt;PI()/2,"beyond breakpoint","interference zone")</f>
+        <v/>
+      </c>
+      <c r="AD30" s="17">
+        <f>IF(AD29&lt;PI()/2,"beyond breakpoint","interference zone")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3512,6 +3799,18 @@
         <f>20*LOG10(AA13/(4*PI()*AA24))</f>
         <v/>
       </c>
+      <c r="AB31" s="15">
+        <f>20*LOG10(AB13/(4*PI()*AB24))</f>
+        <v/>
+      </c>
+      <c r="AC31" s="15">
+        <f>20*LOG10(AC13/(4*PI()*AC24))</f>
+        <v/>
+      </c>
+      <c r="AD31" s="15">
+        <f>20*LOG10(AD13/(4*PI()*AD24))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3626,6 +3925,18 @@
         <f>10*LOG10(1+AA27^2-2*AA27*ABS(COS(AA29)))</f>
         <v/>
       </c>
+      <c r="AB32" s="15">
+        <f>10*LOG10(1+AB27^2-2*AB27*ABS(COS(AB29)))</f>
+        <v/>
+      </c>
+      <c r="AC32" s="15">
+        <f>10*LOG10(1+AC27^2-2*AC27*ABS(COS(AC29)))</f>
+        <v/>
+      </c>
+      <c r="AD32" s="15">
+        <f>10*LOG10(1+AD27^2-2*AD27*ABS(COS(AD29)))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3740,6 +4051,18 @@
         <f>AA31+AA32</f>
         <v/>
       </c>
+      <c r="AB33" s="15">
+        <f>AB31+AB32</f>
+        <v/>
+      </c>
+      <c r="AC33" s="15">
+        <f>AC31+AC32</f>
+        <v/>
+      </c>
+      <c r="AD33" s="15">
+        <f>AD31+AD32</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3831,6 +4154,15 @@
       <c r="AA34" s="16" t="n">
         <v>-1</v>
       </c>
+      <c r="AB34" s="16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC34" s="16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD34" s="16" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3922,6 +4254,15 @@
       <c r="AA35" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="AB35" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC35" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD35" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4013,6 +4354,15 @@
       <c r="AA36" s="16" t="n">
         <v>-10</v>
       </c>
+      <c r="AB36" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC36" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4127,6 +4477,18 @@
         <f>AA20+AA31+AA34</f>
         <v/>
       </c>
+      <c r="AB37" s="15">
+        <f>AB20+AB31+AB34</f>
+        <v/>
+      </c>
+      <c r="AC37" s="15">
+        <f>AC20+AC31+AC34</f>
+        <v/>
+      </c>
+      <c r="AD37" s="15">
+        <f>AD20+AD31+AD34</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4239,6 +4601,18 @@
       </c>
       <c r="AA38" s="15">
         <f>AA20+AA33+AA34+AA35+AA36</f>
+        <v/>
+      </c>
+      <c r="AB38" s="15">
+        <f>AB20+AB33+AB34+AB35+AB36</f>
+        <v/>
+      </c>
+      <c r="AC38" s="15">
+        <f>AC20+AC33+AC34+AC35+AC36</f>
+        <v/>
+      </c>
+      <c r="AD38" s="15">
+        <f>AD20+AD33+AD34+AD35+AD36</f>
         <v/>
       </c>
     </row>
@@ -4274,6 +4648,9 @@
       <c r="Y39" s="7" t="n"/>
       <c r="Z39" s="7" t="n"/>
       <c r="AA39" s="7" t="n"/>
+      <c r="AB39" s="7" t="n"/>
+      <c r="AC39" s="7" t="n"/>
+      <c r="AD39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4365,6 +4742,15 @@
       <c r="AA40" s="16" t="n">
         <v>2</v>
       </c>
+      <c r="AB40" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC40" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD40" s="16" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4452,6 +4838,15 @@
       <c r="AA41" s="11" t="n">
         <v>-0.5</v>
       </c>
+      <c r="AB41" s="11" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="AC41" s="11" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="AD41" s="11" t="n">
+        <v>-0.5</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4566,6 +4961,18 @@
         <f>AA37+AA40+AA41</f>
         <v/>
       </c>
+      <c r="AB42" s="15">
+        <f>AB37+AB40+AB41</f>
+        <v/>
+      </c>
+      <c r="AC42" s="15">
+        <f>AC37+AC40+AC41</f>
+        <v/>
+      </c>
+      <c r="AD42" s="15">
+        <f>AD37+AD40+AD41</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4680,6 +5087,18 @@
         <f>AA38+AA40+AA41</f>
         <v/>
       </c>
+      <c r="AB43" s="15">
+        <f>AB38+AB40+AB41</f>
+        <v/>
+      </c>
+      <c r="AC43" s="15">
+        <f>AC38+AC40+AC41</f>
+        <v/>
+      </c>
+      <c r="AD43" s="15">
+        <f>AD38+AD40+AD41</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4769,6 +5188,15 @@
         <v>-96</v>
       </c>
       <c r="AA44" s="9" t="n">
+        <v>-96</v>
+      </c>
+      <c r="AB44" s="9" t="n">
+        <v>-96</v>
+      </c>
+      <c r="AC44" s="9" t="n">
+        <v>-96</v>
+      </c>
+      <c r="AD44" s="9" t="n">
         <v>-96</v>
       </c>
     </row>
@@ -4892,6 +5320,21 @@
         </is>
       </c>
       <c r="AA45" s="8" t="inlineStr">
+        <is>
+          <t>E01-ML01SP4 datasheet: -96 dBm typ @250 kbps (module with LNA). Measure in T2.</t>
+        </is>
+      </c>
+      <c r="AB45" s="8" t="inlineStr">
+        <is>
+          <t>E01-ML01SP4 datasheet: -96 dBm typ @250 kbps (module with LNA). Measure in T2.</t>
+        </is>
+      </c>
+      <c r="AC45" s="8" t="inlineStr">
+        <is>
+          <t>E01-ML01SP4 datasheet: -96 dBm typ @250 kbps (module with LNA). Measure in T2.</t>
+        </is>
+      </c>
+      <c r="AD45" s="8" t="inlineStr">
         <is>
           <t>E01-ML01SP4 datasheet: -96 dBm typ @250 kbps (module with LNA). Measure in T2.</t>
         </is>
@@ -4929,6 +5372,9 @@
       <c r="Y46" s="7" t="n"/>
       <c r="Z46" s="7" t="n"/>
       <c r="AA46" s="7" t="n"/>
+      <c r="AB46" s="7" t="n"/>
+      <c r="AC46" s="7" t="n"/>
+      <c r="AD46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -5043,6 +5489,18 @@
         <f>AA42-AA44</f>
         <v/>
       </c>
+      <c r="AB47" s="22">
+        <f>AB42-AB44</f>
+        <v/>
+      </c>
+      <c r="AC47" s="22">
+        <f>AC42-AC44</f>
+        <v/>
+      </c>
+      <c r="AD47" s="22">
+        <f>AD42-AD44</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -5157,6 +5615,18 @@
         <f>AA43-AA44</f>
         <v/>
       </c>
+      <c r="AB48" s="23">
+        <f>AB43-AB44</f>
+        <v/>
+      </c>
+      <c r="AC48" s="23">
+        <f>AC43-AC44</f>
+        <v/>
+      </c>
+      <c r="AD48" s="23">
+        <f>AD43-AD44</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -5263,6 +5733,18 @@
       </c>
       <c r="AA49" s="22">
         <f>AA43-AA35+$D$49-AA44</f>
+        <v/>
+      </c>
+      <c r="AB49" s="22">
+        <f>AB43-AB35+$D$49-AB44</f>
+        <v/>
+      </c>
+      <c r="AC49" s="22">
+        <f>AC43-AC35+$D$49-AC44</f>
+        <v/>
+      </c>
+      <c r="AD49" s="22">
+        <f>AD43-AD35+$D$49-AD44</f>
         <v/>
       </c>
     </row>
@@ -5298,6 +5780,9 @@
       <c r="Y50" s="7" t="n"/>
       <c r="Z50" s="7" t="n"/>
       <c r="AA50" s="7" t="n"/>
+      <c r="AB50" s="7" t="n"/>
+      <c r="AC50" s="7" t="n"/>
+      <c r="AD50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -5387,6 +5872,15 @@
         <v>10</v>
       </c>
       <c r="AA51" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB51" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC51" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD51" s="11" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5476,6 +5970,15 @@
       <c r="AA52" s="13" t="n">
         <v>290</v>
       </c>
+      <c r="AB52" s="13" t="n">
+        <v>290</v>
+      </c>
+      <c r="AC52" s="13" t="n">
+        <v>290</v>
+      </c>
+      <c r="AD52" s="13" t="n">
+        <v>290</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5590,6 +6093,18 @@
         <f>AA52*(10^(AA51/10)-1)</f>
         <v/>
       </c>
+      <c r="AB53" s="25">
+        <f>AB52*(10^(AB51/10)-1)</f>
+        <v/>
+      </c>
+      <c r="AC53" s="25">
+        <f>AC52*(10^(AC51/10)-1)</f>
+        <v/>
+      </c>
+      <c r="AD53" s="25">
+        <f>AD52*(10^(AD51/10)-1)</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5679,6 +6194,15 @@
         <v>500</v>
       </c>
       <c r="AA54" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="AB54" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="AC54" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="AD54" s="13" t="n">
         <v>500</v>
       </c>
     </row>
@@ -5768,6 +6292,15 @@
       <c r="AA55" s="13" t="n">
         <v>300</v>
       </c>
+      <c r="AB55" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="AC55" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="AD55" s="13" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5859,6 +6392,15 @@
       <c r="AA56" s="19" t="n">
         <v>1.38</v>
       </c>
+      <c r="AB56" s="19" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="AC56" s="19" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="AD56" s="19" t="n">
+        <v>1.38</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5973,6 +6515,18 @@
         <f>10*LOG10(AA56*(AA55+AA53)*AA54*1000)-230+30</f>
         <v/>
       </c>
+      <c r="AB57" s="15">
+        <f>10*LOG10(AB56*(AB55+AB53)*AB54*1000)-230+30</f>
+        <v/>
+      </c>
+      <c r="AC57" s="15">
+        <f>10*LOG10(AC56*(AC55+AC53)*AC54*1000)-230+30</f>
+        <v/>
+      </c>
+      <c r="AD57" s="15">
+        <f>10*LOG10(AD56*(AD55+AD53)*AD54*1000)-230+30</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -6083,6 +6637,18 @@
         <f>AA44-AA57</f>
         <v/>
       </c>
+      <c r="AB58" s="15">
+        <f>AB44-AB57</f>
+        <v/>
+      </c>
+      <c r="AC58" s="15">
+        <f>AC44-AC57</f>
+        <v/>
+      </c>
+      <c r="AD58" s="15">
+        <f>AD44-AD57</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -6197,6 +6763,18 @@
         <f>AA43-AA57</f>
         <v/>
       </c>
+      <c r="AB59" s="15">
+        <f>AB43-AB57</f>
+        <v/>
+      </c>
+      <c r="AC59" s="15">
+        <f>AC43-AC57</f>
+        <v/>
+      </c>
+      <c r="AD59" s="15">
+        <f>AD43-AD57</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -6436,7 +7014,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>S20: MRM 260 m | E01-ML01DP5 2.4G | 250 kbps, 100 mW FHSS (if Atenea Q3 = yes)</t>
+          <t>S20: MRM 260 m | E01-ML01DP5 2.4G | 250 kbps, 100 mW FHSS (DP5, superseded by S25)</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -6478,6 +7056,42 @@
       <c r="D84" s="4" t="inlineStr">
         <is>
           <t>E01-ML01SP4 @RF_PWR -18 (~+7 dBm, est.), Molex 146153 flex omni 2 dBi in box, 0.5 dB cable</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>S24: SRI 70 m | E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (D-R6)</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>D-R6 draft: adaptive FHSS + LBT, UN-85 a) 20 dBm e.i.r.p.; SP4 at RF_PWR -6/-12 (T0 picks), +17.5 dBm max at the IPEX, omni 3 dBi peak -&gt; &lt;= 20.0 dBm e.i.r.p.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>S25: MRM 260 m | E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (D-R6)</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>D-R6 draft: adaptive FHSS + LBT, UN-85 a) 20 dBm e.i.r.p.; SP4 at RF_PWR -6/-12 (T0 picks), +17.5 dBm max at the IPEX, omni 3 dBi peak -&gt; &lt;= 20.0 dBm e.i.r.p.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>S26: MRM 260 m | E01-ML01SP4 2.4G | 250 kbps, omni, FHSS worst RF_PWR step (D-R6)</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>D-R6 draft, worst RF_PWR step: -6 would overshoot 20 dBm e.i.r.p., so -12 (~+12 dBm at the IPEX) -&gt; ~14.5 dBm e.i.r.p.</t>
         </is>
       </c>
     </row>
@@ -6496,7 +7110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -7141,6 +7755,84 @@
         <v/>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="27">
+        <f>"S24  "&amp;'Link Budget'!AB5&amp;" | "&amp;'Link Budget'!AB6</f>
+        <v/>
+      </c>
+      <c r="B28" s="28">
+        <f>'Link Budget'!AB20+20*LOG10('Link Budget'!AB13/(4*PI()*'Link Budget'!AB24))+10*LOG10(1+'Link Budget'!AB27^2-2*'Link Budget'!AB27*ABS(COS(2*PI()*(SQRT('Link Budget'!AB24^2+(2*B$4)^2)-'Link Budget'!AB24)/'Link Budget'!AB13)))+'Link Budget'!AB34+'Link Budget'!AB35+'Link Budget'!AB36+'Link Budget'!AB40+'Link Budget'!AB41-'Link Budget'!AB44</f>
+        <v/>
+      </c>
+      <c r="C28" s="28">
+        <f>'Link Budget'!AB20+20*LOG10('Link Budget'!AB13/(4*PI()*'Link Budget'!AB24))+10*LOG10(1+'Link Budget'!AB27^2-2*'Link Budget'!AB27*ABS(COS(2*PI()*(SQRT('Link Budget'!AB24^2+(2*C$4)^2)-'Link Budget'!AB24)/'Link Budget'!AB13)))+'Link Budget'!AB34+'Link Budget'!AB35+'Link Budget'!AB36+'Link Budget'!AB40+'Link Budget'!AB41-'Link Budget'!AB44</f>
+        <v/>
+      </c>
+      <c r="D28" s="28">
+        <f>'Link Budget'!AB20+20*LOG10('Link Budget'!AB13/(4*PI()*'Link Budget'!AB24))+10*LOG10(1+'Link Budget'!AB27^2-2*'Link Budget'!AB27*ABS(COS(2*PI()*(SQRT('Link Budget'!AB24^2+(2*D$4)^2)-'Link Budget'!AB24)/'Link Budget'!AB13)))+'Link Budget'!AB34+'Link Budget'!AB35+'Link Budget'!AB36+'Link Budget'!AB40+'Link Budget'!AB41-'Link Budget'!AB44</f>
+        <v/>
+      </c>
+      <c r="E28" s="28">
+        <f>'Link Budget'!AB20+20*LOG10('Link Budget'!AB13/(4*PI()*'Link Budget'!AB24))+10*LOG10(1+'Link Budget'!AB27^2-2*'Link Budget'!AB27*ABS(COS(2*PI()*(SQRT('Link Budget'!AB24^2+(2*E$4)^2)-'Link Budget'!AB24)/'Link Budget'!AB13)))+'Link Budget'!AB34+'Link Budget'!AB35+'Link Budget'!AB36+'Link Budget'!AB40+'Link Budget'!AB41-'Link Budget'!AB44</f>
+        <v/>
+      </c>
+      <c r="F28" s="28">
+        <f>'Link Budget'!AB20+20*LOG10('Link Budget'!AB13/(4*PI()*'Link Budget'!AB24))+10*LOG10(1+'Link Budget'!AB27^2-2*'Link Budget'!AB27*ABS(COS(2*PI()*(SQRT('Link Budget'!AB24^2+(2*F$4)^2)-'Link Budget'!AB24)/'Link Budget'!AB13)))+'Link Budget'!AB34+'Link Budget'!AB35+'Link Budget'!AB36+'Link Budget'!AB40+'Link Budget'!AB41-'Link Budget'!AB44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="27">
+        <f>"S25  "&amp;'Link Budget'!AC5&amp;" | "&amp;'Link Budget'!AC6</f>
+        <v/>
+      </c>
+      <c r="B29" s="28">
+        <f>'Link Budget'!AC20+20*LOG10('Link Budget'!AC13/(4*PI()*'Link Budget'!AC24))+10*LOG10(1+'Link Budget'!AC27^2-2*'Link Budget'!AC27*ABS(COS(2*PI()*(SQRT('Link Budget'!AC24^2+(2*B$4)^2)-'Link Budget'!AC24)/'Link Budget'!AC13)))+'Link Budget'!AC34+'Link Budget'!AC35+'Link Budget'!AC36+'Link Budget'!AC40+'Link Budget'!AC41-'Link Budget'!AC44</f>
+        <v/>
+      </c>
+      <c r="C29" s="28">
+        <f>'Link Budget'!AC20+20*LOG10('Link Budget'!AC13/(4*PI()*'Link Budget'!AC24))+10*LOG10(1+'Link Budget'!AC27^2-2*'Link Budget'!AC27*ABS(COS(2*PI()*(SQRT('Link Budget'!AC24^2+(2*C$4)^2)-'Link Budget'!AC24)/'Link Budget'!AC13)))+'Link Budget'!AC34+'Link Budget'!AC35+'Link Budget'!AC36+'Link Budget'!AC40+'Link Budget'!AC41-'Link Budget'!AC44</f>
+        <v/>
+      </c>
+      <c r="D29" s="28">
+        <f>'Link Budget'!AC20+20*LOG10('Link Budget'!AC13/(4*PI()*'Link Budget'!AC24))+10*LOG10(1+'Link Budget'!AC27^2-2*'Link Budget'!AC27*ABS(COS(2*PI()*(SQRT('Link Budget'!AC24^2+(2*D$4)^2)-'Link Budget'!AC24)/'Link Budget'!AC13)))+'Link Budget'!AC34+'Link Budget'!AC35+'Link Budget'!AC36+'Link Budget'!AC40+'Link Budget'!AC41-'Link Budget'!AC44</f>
+        <v/>
+      </c>
+      <c r="E29" s="28">
+        <f>'Link Budget'!AC20+20*LOG10('Link Budget'!AC13/(4*PI()*'Link Budget'!AC24))+10*LOG10(1+'Link Budget'!AC27^2-2*'Link Budget'!AC27*ABS(COS(2*PI()*(SQRT('Link Budget'!AC24^2+(2*E$4)^2)-'Link Budget'!AC24)/'Link Budget'!AC13)))+'Link Budget'!AC34+'Link Budget'!AC35+'Link Budget'!AC36+'Link Budget'!AC40+'Link Budget'!AC41-'Link Budget'!AC44</f>
+        <v/>
+      </c>
+      <c r="F29" s="28">
+        <f>'Link Budget'!AC20+20*LOG10('Link Budget'!AC13/(4*PI()*'Link Budget'!AC24))+10*LOG10(1+'Link Budget'!AC27^2-2*'Link Budget'!AC27*ABS(COS(2*PI()*(SQRT('Link Budget'!AC24^2+(2*F$4)^2)-'Link Budget'!AC24)/'Link Budget'!AC13)))+'Link Budget'!AC34+'Link Budget'!AC35+'Link Budget'!AC36+'Link Budget'!AC40+'Link Budget'!AC41-'Link Budget'!AC44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="27">
+        <f>"S26  "&amp;'Link Budget'!AD5&amp;" | "&amp;'Link Budget'!AD6</f>
+        <v/>
+      </c>
+      <c r="B30" s="28">
+        <f>'Link Budget'!AD20+20*LOG10('Link Budget'!AD13/(4*PI()*'Link Budget'!AD24))+10*LOG10(1+'Link Budget'!AD27^2-2*'Link Budget'!AD27*ABS(COS(2*PI()*(SQRT('Link Budget'!AD24^2+(2*B$4)^2)-'Link Budget'!AD24)/'Link Budget'!AD13)))+'Link Budget'!AD34+'Link Budget'!AD35+'Link Budget'!AD36+'Link Budget'!AD40+'Link Budget'!AD41-'Link Budget'!AD44</f>
+        <v/>
+      </c>
+      <c r="C30" s="28">
+        <f>'Link Budget'!AD20+20*LOG10('Link Budget'!AD13/(4*PI()*'Link Budget'!AD24))+10*LOG10(1+'Link Budget'!AD27^2-2*'Link Budget'!AD27*ABS(COS(2*PI()*(SQRT('Link Budget'!AD24^2+(2*C$4)^2)-'Link Budget'!AD24)/'Link Budget'!AD13)))+'Link Budget'!AD34+'Link Budget'!AD35+'Link Budget'!AD36+'Link Budget'!AD40+'Link Budget'!AD41-'Link Budget'!AD44</f>
+        <v/>
+      </c>
+      <c r="D30" s="28">
+        <f>'Link Budget'!AD20+20*LOG10('Link Budget'!AD13/(4*PI()*'Link Budget'!AD24))+10*LOG10(1+'Link Budget'!AD27^2-2*'Link Budget'!AD27*ABS(COS(2*PI()*(SQRT('Link Budget'!AD24^2+(2*D$4)^2)-'Link Budget'!AD24)/'Link Budget'!AD13)))+'Link Budget'!AD34+'Link Budget'!AD35+'Link Budget'!AD36+'Link Budget'!AD40+'Link Budget'!AD41-'Link Budget'!AD44</f>
+        <v/>
+      </c>
+      <c r="E30" s="28">
+        <f>'Link Budget'!AD20+20*LOG10('Link Budget'!AD13/(4*PI()*'Link Budget'!AD24))+10*LOG10(1+'Link Budget'!AD27^2-2*'Link Budget'!AD27*ABS(COS(2*PI()*(SQRT('Link Budget'!AD24^2+(2*E$4)^2)-'Link Budget'!AD24)/'Link Budget'!AD13)))+'Link Budget'!AD34+'Link Budget'!AD35+'Link Budget'!AD36+'Link Budget'!AD40+'Link Budget'!AD41-'Link Budget'!AD44</f>
+        <v/>
+      </c>
+      <c r="F30" s="28">
+        <f>'Link Budget'!AD20+20*LOG10('Link Budget'!AD13/(4*PI()*'Link Budget'!AD24))+10*LOG10(1+'Link Budget'!AD27^2-2*'Link Budget'!AD27*ABS(COS(2*PI()*(SQRT('Link Budget'!AD24^2+(2*F$4)^2)-'Link Budget'!AD24)/'Link Budget'!AD13)))+'Link Budget'!AD34+'Link Budget'!AD35+'Link Budget'!AD36+'Link Budget'!AD40+'Link Budget'!AD41-'Link Budget'!AD44</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7152,7 +7844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7827,6 +8519,121 @@
     </row>
     <row r="23"/>
     <row r="24"/>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>D-R6 draft: adaptive FHSS + LBT at 20 dBm e.i.r.p. (only if Atenea Q3 = yes) - nRF24 @250 kbps (row 18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Hop slot (dwell)</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="n">
+        <v>25</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ms</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>One 16-frame SR-ARQ window (~22 ms) + guard; COT must stay &lt; 60 ms (EN 300 328 4.3.1.7.2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Hop + CCA overhead per slot</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ms</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>PLL settle 130 us + RPD needs &gt;= 170 us in RX (the CCA, &gt;= 18 us required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Slots skipped busy (LBT)</t>
+        </is>
+      </c>
+      <c r="B29" s="24" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>ASSUMPTION: campus WiFi + other teams; measure in T14/T17</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Goodput with hopping</t>
+        </is>
+      </c>
+      <c r="B30" s="30">
+        <f>L18*(1-B28/B27)*(1-B29)</f>
+        <v/>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>kbps</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Lines, no compression</t>
+        </is>
+      </c>
+      <c r="B31" s="38">
+        <f>MIN($B$4,INT(B30*1000*$B$5/8/$B$9))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Non-adaptive FHSS at 20 dBm instead (MU &lt;= 10 % -&gt; 10 % duty)</t>
+        </is>
+      </c>
+      <c r="B32" s="30">
+        <f>L18*0.1</f>
+        <v/>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>kbps</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>EN 300 328 4.3.1.6: MU = P/100 mW x DC &lt;= 10 %. Too slow for a 2-min round: hence adaptive (LBT).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A22:P24"/>
@@ -7928,566 +8735,566 @@
       </c>
     </row>
     <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="39" t="inlineStr">
         <is>
           <t>HopeRF RFM69HCW (Semtech SX1231H), 868 MHz variant</t>
         </is>
       </c>
-      <c r="B4" s="38" t="inlineStr">
+      <c r="B4" s="39" t="inlineStr">
         <is>
           <t>433 / 868 / 915 MHz variants</t>
         </is>
       </c>
-      <c r="C4" s="38" t="inlineStr">
+      <c r="C4" s="39" t="inlineStr">
         <is>
           <t>+20 dBm (PA_BOOST); +17 dBm without high-power mode</t>
         </is>
       </c>
-      <c r="D4" s="38" t="inlineStr">
+      <c r="D4" s="39" t="inlineStr">
         <is>
           <t>130 mA @+20; 95 mA @+17</t>
         </is>
       </c>
-      <c r="E4" s="38" t="inlineStr">
+      <c r="E4" s="39" t="inlineStr">
         <is>
           <t>16 mA</t>
         </is>
       </c>
-      <c r="F4" s="38" t="inlineStr">
+      <c r="F4" s="39" t="inlineStr">
         <is>
           <t>-118 dBm @1.2 kbps; -114 @4.8 kbps; -105 @38.4 kbps (FDA 40 kHz). No figure above 38.4 kbps.</t>
         </is>
       </c>
-      <c r="G4" s="38" t="inlineStr">
+      <c r="G4" s="39" t="inlineStr">
         <is>
           <t>300 kbps FSK</t>
         </is>
       </c>
-      <c r="H4" s="38" t="inlineStr">
+      <c r="H4" s="39" t="inlineStr">
         <is>
           <t>+20 dBm limited to 1 % duty cycle (datasheet §3.3.7) -&gt; use +17 dBm for 2-min rounds. 66 B FIFO. No SAW filter.</t>
         </is>
       </c>
-      <c r="I4" s="38" t="inlineStr">
+      <c r="I4" s="39" t="inlineStr">
         <is>
           <t>Proprietary FSK packet radio - LOW risk; confirm on Atenea</t>
         </is>
       </c>
-      <c r="J4" s="38" t="inlineStr">
+      <c r="J4" s="39" t="inlineStr">
         <is>
           <t>SRI/NM/MRM at 868; huge libraries (RadioHead, LowPowerLab)</t>
         </is>
       </c>
-      <c r="K4" s="38" t="inlineStr">
+      <c r="K4" s="39" t="inlineStr">
         <is>
           <t>TO VERIFY (ET to quote Mouser/DigiKey/LCSC)</t>
         </is>
       </c>
-      <c r="L4" s="38" t="inlineStr">
+      <c r="L4" s="39" t="inlineStr">
         <is>
           <t>HopeRF RFM69HCW datasheet v1.1, Tables 2/4/6 and §3.3.7 - https://cdn-shop.adafruit.com/product-files/3076/RFM69HCW-V1.1.pdf</t>
         </is>
       </c>
     </row>
     <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="39" t="inlineStr">
         <is>
           <t>Si4463 modules (e.g. HopeRF RFM26W, NiceRF/Ebyte boards)</t>
         </is>
       </c>
-      <c r="B5" s="38" t="inlineStr">
+      <c r="B5" s="39" t="inlineStr">
         <is>
           <t>142-1050 MHz</t>
         </is>
       </c>
-      <c r="C5" s="38" t="inlineStr">
+      <c r="C5" s="39" t="inlineStr">
         <is>
           <t>+20 dBm</t>
         </is>
       </c>
-      <c r="D5" s="38" t="inlineStr">
+      <c r="D5" s="39" t="inlineStr">
         <is>
           <t>85 mA @+20 dBm, 868 MHz</t>
         </is>
       </c>
-      <c r="E5" s="38" t="inlineStr">
+      <c r="E5" s="39" t="inlineStr">
         <is>
           <t>~10-14 mA (datasheet)</t>
         </is>
       </c>
-      <c r="F5" s="38" t="inlineStr">
+      <c r="F5" s="39" t="inlineStr">
         <is>
           <t>868/915: -109 dBm @40 kbps; -104 @100 kbps; -97 @500 kbps (GFSK, BER 0.1 %); -88 @1 Mbps 4GFSK</t>
         </is>
       </c>
-      <c r="G5" s="38" t="inlineStr">
+      <c r="G5" s="39" t="inlineStr">
         <is>
           <t>500 kbps (G)FSK; 1 Mbps 4GFSK</t>
         </is>
       </c>
-      <c r="H5" s="38" t="inlineStr">
+      <c r="H5" s="39" t="inlineStr">
         <is>
           <t>Best sensitivity + power of the group; no duty-cycle note found. Config via WDS-generated register sets (steeper learning curve).</t>
         </is>
       </c>
-      <c r="I5" s="38" t="inlineStr">
+      <c r="I5" s="39" t="inlineStr">
         <is>
           <t>Proprietary radio, but the datasheet advertises IEEE 802.15.4g PHY support -&gt; LOW-MEDIUM risk; ask Atenea</t>
         </is>
       </c>
-      <c r="J5" s="38" t="inlineStr">
+      <c r="J5" s="39" t="inlineStr">
         <is>
           <t>Strongest 868 option for MRM margin</t>
         </is>
       </c>
-      <c r="K5" s="38" t="inlineStr">
+      <c r="K5" s="39" t="inlineStr">
         <is>
           <t>TO VERIFY</t>
         </is>
       </c>
-      <c r="L5" s="38" t="inlineStr">
+      <c r="L5" s="39" t="inlineStr">
         <is>
           <t>Silicon Labs Si4463/61/60-C datasheet Rev 1.0, Table 3 (RX 915/868 MHz) - https://datasheet.octopart.com/SI4463-C2A-GM-Silicon-Labs-datasheet-78834891.pdf</t>
         </is>
       </c>
     </row>
     <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="39" t="inlineStr">
         <is>
           <t>TI CC1101 modules (e.g. Ebyte E07-M1101D)</t>
         </is>
       </c>
-      <c r="B6" s="38" t="inlineStr">
+      <c r="B6" s="39" t="inlineStr">
         <is>
           <t>300-348 / 387-464 / 779-928 MHz</t>
         </is>
       </c>
-      <c r="C6" s="38" t="inlineStr">
+      <c r="C6" s="39" t="inlineStr">
         <is>
           <t>+12 dBm @868</t>
         </is>
       </c>
-      <c r="D6" s="38" t="inlineStr">
+      <c r="D6" s="39" t="inlineStr">
         <is>
           <t>34 mA @+12 dBm</t>
         </is>
       </c>
-      <c r="E6" s="38" t="inlineStr">
+      <c r="E6" s="39" t="inlineStr">
         <is>
           <t>~15-17 mA</t>
         </is>
       </c>
-      <c r="F6" s="38" t="inlineStr">
+      <c r="F6" s="39" t="inlineStr">
         <is>
           <t>868: -112 dBm @1.2 kBaud; -104 @38.4; -95 @250 (540 kHz filter); -90 @500 kBaud MSK</t>
         </is>
       </c>
-      <c r="G6" s="38" t="inlineStr">
+      <c r="G6" s="39" t="inlineStr">
         <is>
           <t>500 kBaud (600 kbps 4-FSK)</t>
         </is>
       </c>
-      <c r="H6" s="38" t="inlineStr">
+      <c r="H6" s="39" t="inlineStr">
         <is>
           <t>Lowest power of the 868 options. 250 kBaud setting needs 540 kHz filter -&gt; does NOT fit the 250 kHz sub-band; practical ceiling ~100 kbps there.</t>
         </is>
       </c>
-      <c r="I6" s="38" t="inlineStr">
+      <c r="I6" s="39" t="inlineStr">
         <is>
           <t>Proprietary - LOW risk</t>
         </is>
       </c>
-      <c r="J6" s="38" t="inlineStr">
+      <c r="J6" s="39" t="inlineStr">
         <is>
           <t>Fine for SRI; thinner MRM margin</t>
         </is>
       </c>
-      <c r="K6" s="38" t="inlineStr">
+      <c r="K6" s="39" t="inlineStr">
         <is>
           <t>TO VERIFY</t>
         </is>
       </c>
-      <c r="L6" s="38" t="inlineStr">
+      <c r="L6" s="39" t="inlineStr">
         <is>
           <t>TI CC1101 datasheet SWRS061I, Tables 4/7 (868/915 MHz) - https://www.ti.com/lit/ds/symlink/cc1101.pdf</t>
         </is>
       </c>
     </row>
     <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="38" t="inlineStr">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>Nordic nRF24L01+ (and PA/LNA variants)</t>
         </is>
       </c>
-      <c r="B7" s="38" t="inlineStr">
+      <c r="B7" s="39" t="inlineStr">
         <is>
           <t>2.400-2.525 GHz</t>
         </is>
       </c>
-      <c r="C7" s="38" t="inlineStr">
+      <c r="C7" s="39" t="inlineStr">
         <is>
           <t>0 dBm (PA/LNA modules: more, but must be backed off to &lt;=10 dBm e.i.r.p.)</t>
         </is>
       </c>
-      <c r="D7" s="38" t="inlineStr">
+      <c r="D7" s="39" t="inlineStr">
         <is>
           <t>11.3 mA @0 dBm</t>
         </is>
       </c>
-      <c r="E7" s="38" t="inlineStr">
+      <c r="E7" s="39" t="inlineStr">
         <is>
           <t>~12-14 mA</t>
         </is>
       </c>
-      <c r="F7" s="38" t="inlineStr">
+      <c r="F7" s="39" t="inlineStr">
         <is>
           <t>-82 dBm @2 Mbps; -85 @1 Mbps; -94 @250 kbps (BER 0.1 %)</t>
         </is>
       </c>
-      <c r="G7" s="38" t="inlineStr">
+      <c r="G7" s="39" t="inlineStr">
         <is>
           <t>2 Mbps</t>
         </is>
       </c>
-      <c r="H7" s="38" t="inlineStr">
+      <c r="H7" s="39" t="inlineStr">
         <is>
           <t>32 B max payload; auto-ACK/retransmit in hardware (Enhanced ShockBurst). Many clones on the market - buy from a distributor.</t>
         </is>
       </c>
-      <c r="I7" s="38" t="inlineStr">
+      <c r="I7" s="39" t="inlineStr">
         <is>
           <t>Enhanced ShockBurst is Nordic-proprietary - LOW-MEDIUM risk; confirm on Atenea</t>
         </is>
       </c>
-      <c r="J7" s="38" t="inlineStr">
+      <c r="J7" s="39" t="inlineStr">
         <is>
           <t>Speed for SRI; weak margin at 260 m</t>
         </is>
       </c>
-      <c r="K7" s="38" t="inlineStr">
+      <c r="K7" s="39" t="inlineStr">
         <is>
           <t>TO VERIFY</t>
         </is>
       </c>
-      <c r="L7" s="38" t="inlineStr">
+      <c r="L7" s="39" t="inlineStr">
         <is>
           <t>Nordic nRF24L01+ Product Specification v1.0, Tables 7 and 17 - https://www.sparkfun.com/datasheets/Components/SMD/nRF24L01Pluss_Preliminary_Product_Specification_v1_0.pdf</t>
         </is>
       </c>
     </row>
     <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="38" t="inlineStr">
+      <c r="A8" s="39" t="inlineStr">
         <is>
           <t>Not chosen 13-Oct-26 (was the 9-Oct pick): Ebyte E01-ML01DP5 (genuine nRF24L01P + PA/LNA, SMA-K, DIP 2.54 mm)</t>
         </is>
       </c>
-      <c r="B8" s="38" t="inlineStr">
+      <c r="B8" s="39" t="inlineStr">
         <is>
           <t>2.400-2.525 GHz (use &lt;=2483.5)</t>
         </is>
       </c>
-      <c r="C8" s="38" t="inlineStr">
+      <c r="C8" s="39" t="inlineStr">
         <is>
           <t>+20 dBm; ~+7 dBm at RF_PWR -18 (ESTIMATE, PA ~25 dB gain, no bypass)</t>
         </is>
       </c>
-      <c r="D8" s="38" t="inlineStr">
+      <c r="D8" s="39" t="inlineStr">
         <is>
           <t>~120 mA (sister SP4)</t>
         </is>
       </c>
-      <c r="E8" s="38" t="inlineStr">
+      <c r="E8" s="39" t="inlineStr">
         <is>
           <t>~26 mA (sister SP4)</t>
         </is>
       </c>
-      <c r="F8" s="38" t="inlineStr">
+      <c r="F8" s="39" t="inlineStr">
         <is>
           <t>chip -94 dBm @250k / -85 @1M; Ebyte ~-96 @250k for the SP4 (LNA 12 dB, NF 2.5 dB)</t>
         </is>
       </c>
-      <c r="G8" s="38" t="inlineStr">
+      <c r="G8" s="39" t="inlineStr">
         <is>
           <t>2 Mbps</t>
         </is>
       </c>
-      <c r="H8" s="38" t="inlineStr">
+      <c r="H8" s="39" t="inlineStr">
         <is>
           <t>Lowest setting ~+7 dBm: with a 4.5 dBi patch needs ~0.5-3 dB pad for 10 dBm e.i.r.p.; measure (T0). PA/LNA switched inside the module: MCU needs SPI + CE + CSN + IRQ only. 32 B payload.</t>
         </is>
       </c>
-      <c r="I8" s="38" t="inlineStr">
+      <c r="I8" s="39" t="inlineStr">
         <is>
           <t>Proprietary (Enhanced ShockBurst) - LOW-MEDIUM risk; confirm on Atenea</t>
         </is>
       </c>
-      <c r="J8" s="38" t="inlineStr">
+      <c r="J8" s="39" t="inlineStr">
         <is>
           <t>2.4 GHz baseline, all modes</t>
         </is>
       </c>
-      <c r="K8" s="38" t="inlineStr">
+      <c r="K8" s="39" t="inlineStr">
         <is>
           <t>~US$3.9 (Tindie, EBYTE store) - VERIFY lead time to Spain</t>
         </is>
       </c>
-      <c r="L8" s="38" t="inlineStr">
+      <c r="L8" s="39" t="inlineStr">
         <is>
           <t>https://www.cdebyte.com/products/E01-ML01DP5 ; https://voltiq.ru/datasheets/ebyte/E01-ML01SP4.pdf</t>
         </is>
       </c>
     </row>
     <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="38" t="inlineStr">
+      <c r="A9" s="39" t="inlineStr">
         <is>
           <t>DECIDED 13-Oct-26: Ebyte E01-ML01SP4 (genuine nRF24L01P + PA/LNA, SMD 14.85 x 18 mm, IPEX)</t>
         </is>
       </c>
-      <c r="B9" s="38" t="inlineStr">
+      <c r="B9" s="39" t="inlineStr">
         <is>
           <t>2.4 GHz</t>
         </is>
       </c>
-      <c r="C9" s="38" t="inlineStr">
+      <c r="C9" s="39" t="inlineStr">
         <is>
           <t>+20 dBm max; ~+2..+7 dBm at RF_PWR -18 (ESTIMATE, T0)</t>
         </is>
       </c>
-      <c r="D9" s="38" t="inlineStr">
+      <c r="D9" s="39" t="inlineStr">
         <is>
           <t>120 mA</t>
         </is>
       </c>
-      <c r="E9" s="38" t="inlineStr">
+      <c r="E9" s="39" t="inlineStr">
         <is>
           <t>26 mA</t>
         </is>
       </c>
-      <c r="F9" s="38" t="inlineStr">
+      <c r="F9" s="39" t="inlineStr">
         <is>
           <t>-96 dBm typ @250k (datasheet)</t>
         </is>
       </c>
-      <c r="G9" s="38" t="inlineStr">
+      <c r="G9" s="39" t="inlineStr">
         <is>
           <t>2 Mbps</t>
         </is>
       </c>
-      <c r="H9" s="38" t="inlineStr">
+      <c r="H9" s="39" t="inlineStr">
         <is>
           <t>10 pads, 1.27 mm pitch: VCC, CE, CSN, SCK, MOSI, MISO, IRQ, 3x GND. 2.0-3.6 V. IPEX: the Molex flex omni plugs in directly. Needs a breakout from the first bench test (QM module = final).</t>
         </is>
       </c>
-      <c r="I9" s="38" t="inlineStr">
+      <c r="I9" s="39" t="inlineStr">
         <is>
           <t>Proprietary (Enhanced ShockBurst) - LOW-MEDIUM risk; confirm on Atenea</t>
         </is>
       </c>
-      <c r="J9" s="38" t="inlineStr">
+      <c r="J9" s="39" t="inlineStr">
         <is>
           <t>2.4 GHz baseline with one omni</t>
         </is>
       </c>
-      <c r="K9" s="38" t="inlineStr">
+      <c r="K9" s="39" t="inlineStr">
         <is>
           <t>VERIFY</t>
         </is>
       </c>
-      <c r="L9" s="38" t="inlineStr">
+      <c r="L9" s="39" t="inlineStr">
         <is>
           <t>https://voltiq.ru/datasheets/ebyte/E01-ML01SP4.pdf</t>
         </is>
       </c>
     </row>
     <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="38" t="inlineStr">
+      <c r="A10" s="39" t="inlineStr">
         <is>
           <t>EXCLUDE: Ebyte E01C-* and no-name 'nRF24L01+PA+LNA' boards</t>
         </is>
       </c>
-      <c r="B10" s="38" t="inlineStr">
+      <c r="B10" s="39" t="inlineStr">
         <is>
           <t>2.4 GHz</t>
         </is>
       </c>
-      <c r="C10" s="38" t="inlineStr"/>
-      <c r="D10" s="38" t="inlineStr"/>
-      <c r="E10" s="38" t="inlineStr"/>
-      <c r="F10" s="38" t="inlineStr"/>
-      <c r="G10" s="38" t="inlineStr"/>
-      <c r="H10" s="38" t="inlineStr">
+      <c r="C10" s="39" t="inlineStr"/>
+      <c r="D10" s="39" t="inlineStr"/>
+      <c r="E10" s="39" t="inlineStr"/>
+      <c r="F10" s="39" t="inlineStr"/>
+      <c r="G10" s="39" t="inlineStr"/>
+      <c r="H10" s="39" t="inlineStr">
         <is>
           <t>Ebyte's own E01C manual states the chip is a Si24R1 clone (worse receiver, selectivity unknown)</t>
         </is>
       </c>
-      <c r="I10" s="38" t="inlineStr"/>
-      <c r="J10" s="38" t="inlineStr">
+      <c r="I10" s="39" t="inlineStr"/>
+      <c r="J10" s="39" t="inlineStr">
         <is>
           <t>Do not buy (bench only)</t>
         </is>
       </c>
-      <c r="K10" s="38" t="inlineStr"/>
-      <c r="L10" s="38" t="inlineStr">
+      <c r="K10" s="39" t="inlineStr"/>
+      <c r="L10" s="39" t="inlineStr">
         <is>
           <t>https://atta.szlcsc.com/upload/public/pdf/source/20220121/F2AB78B6B3F0E91D6E5268DDE53AA4EA.pdf</t>
         </is>
       </c>
     </row>
     <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="38" t="inlineStr">
+      <c r="A11" s="39" t="inlineStr">
         <is>
           <t>TI CC2500</t>
         </is>
       </c>
-      <c r="B11" s="38" t="inlineStr">
+      <c r="B11" s="39" t="inlineStr">
         <is>
           <t>2.400-2.4835 GHz</t>
         </is>
       </c>
-      <c r="C11" s="38" t="inlineStr">
+      <c r="C11" s="39" t="inlineStr">
         <is>
           <t>+1 dBm</t>
         </is>
       </c>
-      <c r="D11" s="38" t="inlineStr">
+      <c r="D11" s="39" t="inlineStr">
         <is>
           <t>21.5 mA @+1 dBm</t>
         </is>
       </c>
-      <c r="E11" s="38" t="inlineStr">
+      <c r="E11" s="39" t="inlineStr">
         <is>
           <t>~13-17 mA</t>
         </is>
       </c>
-      <c r="F11" s="38" t="inlineStr">
+      <c r="F11" s="39" t="inlineStr">
         <is>
           <t>-104 dBm @2.4 kBaud; -99 @10 kBaud; -89 @250 kBaud; -83 @500 kBaud</t>
         </is>
       </c>
-      <c r="G11" s="38" t="inlineStr">
+      <c r="G11" s="39" t="inlineStr">
         <is>
           <t>500 kBaud</t>
         </is>
       </c>
-      <c r="H11" s="38" t="inlineStr">
+      <c r="H11" s="39" t="inlineStr">
         <is>
           <t>Similar class to nRF24 with more modulation control.</t>
         </is>
       </c>
-      <c r="I11" s="38" t="inlineStr">
+      <c r="I11" s="39" t="inlineStr">
         <is>
           <t>Proprietary - LOW risk</t>
         </is>
       </c>
-      <c r="J11" s="38" t="inlineStr">
+      <c r="J11" s="39" t="inlineStr">
         <is>
           <t>Alternative 2.4 GHz option</t>
         </is>
       </c>
-      <c r="K11" s="38" t="inlineStr">
+      <c r="K11" s="39" t="inlineStr">
         <is>
           <t>TO VERIFY</t>
         </is>
       </c>
-      <c r="L11" s="38" t="inlineStr">
+      <c r="L11" s="39" t="inlineStr">
         <is>
           <t>TI CC2500 datasheet, RF receive section - https://www.ti.com/lit/ds/symlink/cc2500.pdf</t>
         </is>
       </c>
     </row>
     <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="38" t="inlineStr">
+      <c r="A12" s="39" t="inlineStr">
         <is>
           <t>EXCLUDE: LoRa chips (SX127x/RFM95, SX126x, SX1280, LLCC68)</t>
         </is>
       </c>
-      <c r="B12" s="38" t="inlineStr">
+      <c r="B12" s="39" t="inlineStr">
         <is>
           <t>433/868/2.4 GHz</t>
         </is>
       </c>
-      <c r="C12" s="38" t="inlineStr"/>
-      <c r="D12" s="38" t="inlineStr"/>
-      <c r="E12" s="38" t="inlineStr"/>
-      <c r="F12" s="38" t="inlineStr"/>
-      <c r="G12" s="38" t="inlineStr"/>
-      <c r="H12" s="38" t="inlineStr"/>
-      <c r="I12" s="38" t="inlineStr">
+      <c r="C12" s="39" t="inlineStr"/>
+      <c r="D12" s="39" t="inlineStr"/>
+      <c r="E12" s="39" t="inlineStr"/>
+      <c r="F12" s="39" t="inlineStr"/>
+      <c r="G12" s="39" t="inlineStr"/>
+      <c r="H12" s="39" t="inlineStr"/>
+      <c r="I12" s="39" t="inlineStr">
         <is>
           <t>LoRa is named as banned on the Session 1 spec slide; even FSK-only use of a LoRa chip is a compliance risk</t>
         </is>
       </c>
-      <c r="J12" s="38" t="inlineStr">
+      <c r="J12" s="39" t="inlineStr">
         <is>
           <t>Do not buy</t>
         </is>
       </c>
-      <c r="K12" s="38" t="inlineStr"/>
-      <c r="L12" s="38" t="inlineStr">
+      <c r="K12" s="39" t="inlineStr"/>
+      <c r="L12" s="39" t="inlineStr">
         <is>
           <t>Session #1 slide 'Transceiver Specs (I)'</t>
         </is>
       </c>
     </row>
     <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="38" t="inlineStr">
+      <c r="A13" s="39" t="inlineStr">
         <is>
           <t>EXCLUDE: radio SoCs (CC1310/CC1312, nRF52, ESP32, STM32WL...)</t>
         </is>
       </c>
-      <c r="B13" s="38" t="inlineStr"/>
-      <c r="C13" s="38" t="inlineStr"/>
-      <c r="D13" s="38" t="inlineStr"/>
-      <c r="E13" s="38" t="inlineStr"/>
-      <c r="F13" s="38" t="inlineStr"/>
-      <c r="G13" s="38" t="inlineStr"/>
-      <c r="H13" s="38" t="inlineStr"/>
-      <c r="I13" s="38" t="inlineStr">
+      <c r="B13" s="39" t="inlineStr"/>
+      <c r="C13" s="39" t="inlineStr"/>
+      <c r="D13" s="39" t="inlineStr"/>
+      <c r="E13" s="39" t="inlineStr"/>
+      <c r="F13" s="39" t="inlineStr"/>
+      <c r="G13" s="39" t="inlineStr"/>
+      <c r="H13" s="39" t="inlineStr"/>
+      <c r="I13" s="39" t="inlineStr">
         <is>
           <t>Contain a microprocessor (second micro module) and/or BLE/ZigBee/LoRa stacks</t>
         </is>
       </c>
-      <c r="J13" s="38" t="inlineStr">
+      <c r="J13" s="39" t="inlineStr">
         <is>
           <t>Do not buy</t>
         </is>
       </c>
-      <c r="K13" s="38" t="inlineStr"/>
-      <c r="L13" s="38" t="inlineStr">
+      <c r="K13" s="39" t="inlineStr"/>
+      <c r="L13" s="39" t="inlineStr">
         <is>
           <t>Rules PDF: 'one but only one module including a microprocessor'; standard-protocol ban</t>
         </is>
       </c>
     </row>
     <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="38" t="inlineStr">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>EXCLUDE: 915 MHz (US) module variants</t>
         </is>
       </c>
-      <c r="B14" s="38" t="inlineStr">
+      <c r="B14" s="39" t="inlineStr">
         <is>
           <t>902-928 MHz</t>
         </is>
       </c>
-      <c r="C14" s="38" t="inlineStr"/>
-      <c r="D14" s="38" t="inlineStr"/>
-      <c r="E14" s="38" t="inlineStr"/>
-      <c r="F14" s="38" t="inlineStr"/>
-      <c r="G14" s="38" t="inlineStr"/>
-      <c r="H14" s="38" t="inlineStr"/>
-      <c r="I14" s="38" t="inlineStr">
+      <c r="C14" s="39" t="inlineStr"/>
+      <c r="D14" s="39" t="inlineStr"/>
+      <c r="E14" s="39" t="inlineStr"/>
+      <c r="F14" s="39" t="inlineStr"/>
+      <c r="G14" s="39" t="inlineStr"/>
+      <c r="H14" s="39" t="inlineStr"/>
+      <c r="I14" s="39" t="inlineStr">
         <is>
           <t>915-921 MHz is mobile/GSM-R spectrum in Spain (CNAF UN-40), not SRD</t>
         </is>
       </c>
-      <c r="J14" s="38" t="inlineStr">
+      <c r="J14" s="39" t="inlineStr">
         <is>
           <t>Buy 868 variants only</t>
         </is>
       </c>
-      <c r="K14" s="38" t="inlineStr"/>
-      <c r="L14" s="38" t="inlineStr">
+      <c r="K14" s="39" t="inlineStr"/>
+      <c r="L14" s="39" t="inlineStr">
         <is>
           <t>CNAF 2017 (Orden ETU/1033/2017), notas UN - https://www.boe.es/buscar/doc.php?id=BOE-A-2017-12318</t>
         </is>
@@ -8568,321 +9375,321 @@
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="39" t="inlineStr">
+      <c r="A5" s="40" t="inlineStr">
         <is>
           <t>433.050-434.790 MHz</t>
         </is>
       </c>
-      <c r="B5" s="39" t="inlineStr">
+      <c r="B5" s="40" t="inlineStr">
         <is>
           <t>UN-30</t>
         </is>
       </c>
-      <c r="C5" s="39" t="inlineStr">
+      <c r="C5" s="40" t="inlineStr">
         <is>
           <t>1 mW e.r.p. (-13 dBm/10 kHz)</t>
         </is>
       </c>
-      <c r="D5" s="39" t="inlineStr">
+      <c r="D5" s="40" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="E5" s="39" t="inlineStr">
+      <c r="E5" s="40" t="inlineStr">
         <is>
           <t>Yes, but 1 mW</t>
         </is>
       </c>
-      <c r="F5" s="39" t="inlineStr">
+      <c r="F5" s="40" t="inlineStr">
         <is>
           <t>1.74 MHz</t>
         </is>
       </c>
-      <c r="G5" s="39" t="inlineStr">
+      <c r="G5" s="40" t="inlineStr">
         <is>
           <t>Too weak.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="39" t="inlineStr">
+      <c r="A6" s="40" t="inlineStr">
         <is>
           <t>433.050-434.040 MHz</t>
         </is>
       </c>
-      <c r="B6" s="39" t="inlineStr">
+      <c r="B6" s="40" t="inlineStr">
         <is>
           <t>UN-30</t>
         </is>
       </c>
-      <c r="C6" s="39" t="inlineStr">
+      <c r="C6" s="40" t="inlineStr">
         <is>
           <t>10 mW e.r.p.</t>
         </is>
       </c>
-      <c r="D6" s="39" t="inlineStr">
+      <c r="D6" s="40" t="inlineStr">
         <is>
           <t>duty cycle &lt;= 10 %</t>
         </is>
       </c>
-      <c r="E6" s="39" t="inlineStr">
+      <c r="E6" s="40" t="inlineStr">
         <is>
           <t>Yes (120 s &lt; 360 s/h)</t>
         </is>
       </c>
-      <c r="F6" s="39" t="inlineStr">
+      <c r="F6" s="40" t="inlineStr">
         <is>
           <t>0.99 MHz</t>
         </is>
       </c>
-      <c r="G6" s="39" t="inlineStr">
+      <c r="G6" s="40" t="inlineStr">
         <is>
           <t>λ/4 = 17 cm: does not fit the 15x15x7 cm box without heavy shortening.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="40" t="inlineStr">
         <is>
           <t>868.000-868.600 MHz</t>
         </is>
       </c>
-      <c r="B7" s="39" t="inlineStr">
+      <c r="B7" s="40" t="inlineStr">
         <is>
           <t>UN-39</t>
         </is>
       </c>
-      <c r="C7" s="39" t="inlineStr">
+      <c r="C7" s="40" t="inlineStr">
         <is>
           <t>25 mW e.r.p.</t>
         </is>
       </c>
-      <c r="D7" s="39" t="inlineStr">
+      <c r="D7" s="40" t="inlineStr">
         <is>
           <t>LBT+AFA (EN 300 220) or duty cycle &lt;= 1 %</t>
         </is>
       </c>
-      <c r="E7" s="39" t="inlineStr">
+      <c r="E7" s="40" t="inlineStr">
         <is>
           <t>No (1 % = 36 s/h)</t>
         </is>
       </c>
-      <c r="F7" s="39" t="inlineStr">
+      <c r="F7" s="40" t="inlineStr">
         <is>
           <t>600 kHz</t>
         </is>
       </c>
-      <c r="G7" s="39" t="inlineStr"/>
+      <c r="G7" s="40" t="inlineStr"/>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="40" t="inlineStr">
         <is>
           <t>868.700-869.200 MHz</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
           <t>UN-39</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="40" t="inlineStr">
         <is>
           <t>25 mW e.r.p.</t>
         </is>
       </c>
-      <c r="D8" s="39" t="inlineStr">
+      <c r="D8" s="40" t="inlineStr">
         <is>
           <t>LBT+AFA or duty cycle &lt;= 0.1 %</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="40" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
+      <c r="F8" s="40" t="inlineStr">
         <is>
           <t>500 kHz</t>
         </is>
       </c>
-      <c r="G8" s="39" t="inlineStr"/>
+      <c r="G8" s="40" t="inlineStr"/>
     </row>
     <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="41" t="inlineStr">
         <is>
           <t>869.400-869.650 MHz</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="41" t="inlineStr">
         <is>
           <t>UN-39</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="41" t="inlineStr">
         <is>
           <t>500 mW e.r.p.</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="41" t="inlineStr">
         <is>
           <t>LBT+AFA or duty cycle &lt;= 10 %</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="E9" s="41" t="inlineStr">
         <is>
           <t>YES (120 s &lt; 360 s/h)</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="41" t="inlineStr">
         <is>
           <t>250 kHz</t>
         </is>
       </c>
-      <c r="G9" s="40" t="inlineStr">
+      <c r="G9" s="41" t="inlineStr">
         <is>
           <t>THE 868 option. 25 kHz channelisation, but the whole band may be one high-speed data channel. One 120 s SRI + one 120 s MRM = 240 s/h for the TX device: compliant.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="39" t="inlineStr">
+      <c r="A10" s="40" t="inlineStr">
         <is>
           <t>869.700-870.000 MHz</t>
         </is>
       </c>
-      <c r="B10" s="39" t="inlineStr">
+      <c r="B10" s="40" t="inlineStr">
         <is>
           <t>UN-39</t>
         </is>
       </c>
-      <c r="C10" s="39" t="inlineStr">
+      <c r="C10" s="40" t="inlineStr">
         <is>
           <t>5 mW e.r.p. (no DC) / 25 mW (DC &lt;= 1 %)</t>
         </is>
       </c>
-      <c r="D10" s="39" t="inlineStr"/>
-      <c r="E10" s="39" t="inlineStr">
+      <c r="D10" s="40" t="inlineStr"/>
+      <c r="E10" s="40" t="inlineStr">
         <is>
           <t>5 mW only</t>
         </is>
       </c>
-      <c r="F10" s="39" t="inlineStr">
+      <c r="F10" s="40" t="inlineStr">
         <is>
           <t>300 kHz</t>
         </is>
       </c>
-      <c r="G10" s="39" t="inlineStr">
+      <c r="G10" s="40" t="inlineStr">
         <is>
           <t>Low power.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="40" t="inlineStr">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>2400-2483.5 MHz</t>
         </is>
       </c>
-      <c r="B11" s="40" t="inlineStr">
+      <c r="B11" s="41" t="inlineStr">
         <is>
           <t>UN-85 b)</t>
         </is>
       </c>
-      <c r="C11" s="40" t="inlineStr">
+      <c r="C11" s="41" t="inlineStr">
         <is>
           <t>10 mW e.i.r.p.</t>
         </is>
       </c>
-      <c r="D11" s="40" t="inlineStr">
+      <c r="D11" s="41" t="inlineStr">
         <is>
           <t>none (generic SRD, EN 300 440)</t>
         </is>
       </c>
-      <c r="E11" s="40" t="inlineStr">
+      <c r="E11" s="41" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F11" s="40" t="inlineStr">
+      <c r="F11" s="41" t="inlineStr">
         <is>
           <t>83.5 MHz</t>
         </is>
       </c>
-      <c r="G11" s="40" t="inlineStr">
+      <c r="G11" s="41" t="inlineStr">
         <is>
           <t>Room for every team on its own channel (MRM). Campus WiFi/BT share the band.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="39" t="inlineStr">
+      <c r="A12" s="41" t="inlineStr">
         <is>
           <t>2400-2483.5 MHz</t>
         </is>
       </c>
-      <c r="B12" s="39" t="inlineStr">
+      <c r="B12" s="41" t="inlineStr">
         <is>
           <t>UN-85 a)</t>
         </is>
       </c>
-      <c r="C12" s="39" t="inlineStr">
+      <c r="C12" s="41" t="inlineStr">
         <is>
           <t>100 mW e.i.r.p.; 100 mW/100 kHz FHSS, 10 mW/MHz other</t>
         </is>
       </c>
-      <c r="D12" s="39" t="inlineStr">
+      <c r="D12" s="41" t="inlineStr">
         <is>
           <t>mitigation techniques (EN 300 328) mandatory</t>
         </is>
       </c>
-      <c r="E12" s="39" t="inlineStr">
+      <c r="E12" s="41" t="inlineStr">
         <is>
           <t>Yes, if mitigation implemented</t>
         </is>
       </c>
-      <c r="F12" s="39" t="inlineStr">
+      <c r="F12" s="41" t="inlineStr">
         <is>
           <t>83.5 MHz</t>
         </is>
       </c>
-      <c r="G12" s="39" t="inlineStr">
-        <is>
-          <t>Wideband data/RLAN class. Whether a student FHSS/LBT design qualifies is a question for Atenea.</t>
+      <c r="G12" s="41" t="inlineStr">
+        <is>
+          <t>D-R6 draft (16-Oct): SRI/MRM as adaptive FHSS + LBT (EN 300 328 4.3.1.7.2: &gt;= 15 hop channels over &gt;= 70 % of the band, CCA at -70 dBm/MHz, COT &lt; 60 ms). A non-hopping narrowband radio gets nothing here (10 mW/MHz = 10 dBm in our &lt; 1 MHz). Non-adaptive FHSS: MU &lt;= 10 % (10 % duty at 20 dBm). Needs Atenea Q3 = yes.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="39" t="inlineStr">
+      <c r="A13" s="40" t="inlineStr">
         <is>
           <t>5725-5875 MHz</t>
         </is>
       </c>
-      <c r="B13" s="39" t="inlineStr">
+      <c r="B13" s="40" t="inlineStr">
         <is>
           <t>UN-130</t>
         </is>
       </c>
-      <c r="C13" s="39" t="inlineStr">
+      <c r="C13" s="40" t="inlineStr">
         <is>
           <t>25 mW e.i.r.p.</t>
         </is>
       </c>
-      <c r="D13" s="39" t="inlineStr">
+      <c r="D13" s="40" t="inlineStr">
         <is>
           <t>none (generic SRD, EN 300 440)</t>
         </is>
       </c>
-      <c r="E13" s="39" t="inlineStr">
+      <c r="E13" s="40" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F13" s="39" t="inlineStr">
+      <c r="F13" s="40" t="inlineStr">
         <is>
           <t>150 MHz</t>
         </is>
       </c>
-      <c r="G13" s="39" t="inlineStr">
+      <c r="G13" s="40" t="inlineStr">
         <is>
           <t>Few cheap non-WiFi modules; higher path loss and container loss. Not shortlisted.</t>
         </is>

</xml_diff>

<commit_message>
Make 20 dBm hopping (D-R6) the SRI/MRM baseline: a professor approved 20 dBm e.i.r.p.
- hop guard widened to +-5 MHz (27 channels, nearest hop 6 MHz, C/I -50 dB): at 5 MHz our 20 dBm
  would drown a 10 mW neighbour; near-far printout: >= 15 m from 10 mW teams' boxes at MRM
- linkbudget/workbook: S24-S26 = SRI/MRM baseline, S23 = NM at 10 mW, S21-S22 = 10 mW fallback (0 dB diff)
- phy_config: TEAM_FHSS = SRI/MRM, TEAM_250K = Quick Mode/bench/fallback; fw 194 checks; sim 13/13
- docs: DECISIONS D-R6 baseline, TEST_PLAN v0.5, Atenea Q3 = written confirmation, handoff, READMEs, CLAUDE.md
- pages: brief v0.7, hardware v0.4.2, protocol v0.3.3 republished; PDFs re-exported

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MU9yLRr2JqK4PHEE7hWEta
</commit_message>
<xml_diff>
--- a/radio/MTP-F26_TeamC_Radio_LinkBudget.xlsx
+++ b/radio/MTP-F26_TeamC_Radio_LinkBudget.xlsx
@@ -593,7 +593,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>S21-S23 = 2.4 GHz baseline (E01-ML01SP4 + one omni, 10 mW e.i.r.p.). S24-S26 = D-R6 draft: same hardware as adaptive FHSS + LBT at 20 dBm e.i.r.p. (UN-85 a), only if Atenea Q3 = yes.</t>
+          <t>Baseline (16-Oct): S24-S26 = SRI/MRM on the E01-ML01SP4 + one omni as adaptive FHSS + LBT at &lt;= 20 dBm e.i.r.p. (UN-85 a, D-R6; S26 = RF_PWR -12 until T0). S23 = NM at 10 mW on one channel. S21-S22 = the 10 mW fixed-channel fallback (and Quick Mode).</t>
         </is>
       </c>
     </row>
@@ -1221,32 +1221,32 @@
       </c>
       <c r="Y6" s="8" t="inlineStr">
         <is>
-          <t>E01-ML01SP4 2.4G | 250 kbps, omni (2.4 baseline)</t>
+          <t>E01-ML01SP4 2.4G | 250 kbps, omni, 10 mW fixed (QM/fallback)</t>
         </is>
       </c>
       <c r="Z6" s="8" t="inlineStr">
         <is>
-          <t>E01-ML01SP4 2.4G | 250 kbps, omni (2.4 baseline)</t>
+          <t>E01-ML01SP4 2.4G | 250 kbps, omni, 10 mW fixed (fallback)</t>
         </is>
       </c>
       <c r="AA6" s="8" t="inlineStr">
         <is>
-          <t>E01-ML01SP4 2.4G | 250 kbps, -10 dB obstr., omni (2.4 baseline)</t>
+          <t>E01-ML01SP4 2.4G | 250 kbps, -10 dB obstr., omni, 10 mW (baseline)</t>
         </is>
       </c>
       <c r="AB6" s="8" t="inlineStr">
         <is>
-          <t>E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (D-R6)</t>
+          <t>E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (baseline)</t>
         </is>
       </c>
       <c r="AC6" s="8" t="inlineStr">
         <is>
-          <t>E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (D-R6)</t>
+          <t>E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (baseline)</t>
         </is>
       </c>
       <c r="AD6" s="8" t="inlineStr">
         <is>
-          <t>E01-ML01SP4 2.4G | 250 kbps, omni, FHSS worst RF_PWR step (D-R6)</t>
+          <t>E01-ML01SP4 2.4G | 250 kbps, omni, FHSS at RF_PWR -12 (until T0)</t>
         </is>
       </c>
     </row>
@@ -7026,7 +7026,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>S21: SRI 70 m | E01-ML01SP4 2.4G | 250 kbps, omni (2.4 baseline)</t>
+          <t>S21: SRI 70 m | E01-ML01SP4 2.4G | 250 kbps, omni, 10 mW fixed (QM/fallback)</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -7038,7 +7038,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>S22: MRM 260 m | E01-ML01SP4 2.4G | 250 kbps, omni (2.4 baseline)</t>
+          <t>S22: MRM 260 m | E01-ML01SP4 2.4G | 250 kbps, omni, 10 mW fixed (fallback)</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -7050,7 +7050,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>S23: NM hop 100 m | E01-ML01SP4 2.4G | 250 kbps, -10 dB obstr., omni (2.4 baseline)</t>
+          <t>S23: NM hop 100 m | E01-ML01SP4 2.4G | 250 kbps, -10 dB obstr., omni, 10 mW (baseline)</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -7062,36 +7062,36 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>S24: SRI 70 m | E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (D-R6)</t>
+          <t>S24: SRI 70 m | E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (baseline)</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>D-R6 draft: adaptive FHSS + LBT, UN-85 a) 20 dBm e.i.r.p.; SP4 at RF_PWR -6/-12 (T0 picks), +17.5 dBm max at the IPEX, omni 3 dBi peak -&gt; &lt;= 20.0 dBm e.i.r.p.</t>
+          <t>D-R6 baseline: adaptive FHSS + LBT, UN-85 a) 20 dBm e.i.r.p.; SP4 at RF_PWR -6/-12 (T0 picks), +17.5 dBm max at the IPEX, omni 3 dBi peak -&gt; &lt;= 20.0 dBm e.i.r.p.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>S25: MRM 260 m | E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (D-R6)</t>
+          <t>S25: MRM 260 m | E01-ML01SP4 2.4G | 250 kbps, omni, FHSS 20 dBm (baseline)</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>D-R6 draft: adaptive FHSS + LBT, UN-85 a) 20 dBm e.i.r.p.; SP4 at RF_PWR -6/-12 (T0 picks), +17.5 dBm max at the IPEX, omni 3 dBi peak -&gt; &lt;= 20.0 dBm e.i.r.p.</t>
+          <t>D-R6 baseline: adaptive FHSS + LBT, UN-85 a) 20 dBm e.i.r.p.; SP4 at RF_PWR -6/-12 (T0 picks), +17.5 dBm max at the IPEX, omni 3 dBi peak -&gt; &lt;= 20.0 dBm e.i.r.p.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>S26: MRM 260 m | E01-ML01SP4 2.4G | 250 kbps, omni, FHSS worst RF_PWR step (D-R6)</t>
+          <t>S26: MRM 260 m | E01-ML01SP4 2.4G | 250 kbps, omni, FHSS at RF_PWR -12 (until T0)</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>D-R6 draft, worst RF_PWR step: -6 would overshoot 20 dBm e.i.r.p., so -12 (~+12 dBm at the IPEX) -&gt; ~14.5 dBm e.i.r.p.</t>
+          <t>D-R6, worst RF_PWR step: -6 would overshoot 20 dBm e.i.r.p., so -12 (~+12 dBm at the IPEX) -&gt; ~14.5 dBm e.i.r.p.</t>
         </is>
       </c>
     </row>
@@ -8522,7 +8522,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>D-R6 draft: adaptive FHSS + LBT at 20 dBm e.i.r.p. (only if Atenea Q3 = yes) - nRF24 @250 kbps (row 18)</t>
+          <t>SRI/MRM baseline (D-R6): adaptive FHSS + LBT at &lt;= 20 dBm e.i.r.p. - nRF24 @250 kbps (row 18)</t>
         </is>
       </c>
     </row>
@@ -9654,7 +9654,7 @@
       </c>
       <c r="G12" s="41" t="inlineStr">
         <is>
-          <t>D-R6 draft (16-Oct): SRI/MRM as adaptive FHSS + LBT (EN 300 328 4.3.1.7.2: &gt;= 15 hop channels over &gt;= 70 % of the band, CCA at -70 dBm/MHz, COT &lt; 60 ms). A non-hopping narrowband radio gets nothing here (10 mW/MHz = 10 dBm in our &lt; 1 MHz). Non-adaptive FHSS: MU &lt;= 10 % (10 % duty at 20 dBm). Needs Atenea Q3 = yes.</t>
+          <t>SRI/MRM baseline since 16-Oct (D-R6, a professor approved 20 dBm): adaptive FHSS + LBT (EN 300 328 4.3.1.7.2: &gt;= 15 hop channels over &gt;= 70 % of the band, CCA at -70 dBm/MHz, COT &lt; 60 ms). A non-hopping narrowband radio gets nothing here (10 mW/MHz = 10 dBm in our &lt; 1 MHz). Non-adaptive FHSS: MU &lt;= 10 % (10 % duty at 20 dBm). Written confirmation requested on Atenea (Q3).</t>
         </is>
       </c>
     </row>

</xml_diff>